<commit_message>
Add WK-30 VOC data
</commit_message>
<xml_diff>
--- a/VOC_data.xlsx
+++ b/VOC_data.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,46 +425,46 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H289"/>
+  <dimension ref="A1:H297"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Wbr Carrier Group</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Year ID</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Vendor Code</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Vendor Name</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Week ID</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>DEA %</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Unpadded DEA %</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>PDD Shipment #</t>
         </is>
@@ -9672,6 +9684,262 @@
       </c>
       <c r="H289" t="n">
         <v>8923</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>VOC</t>
+        </is>
+      </c>
+      <c r="B290" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>0V6VN</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>JustFoodForDogs -- Dropship</t>
+        </is>
+      </c>
+      <c r="E290" t="n">
+        <v>202630</v>
+      </c>
+      <c r="F290" t="n">
+        <v>0.965</v>
+      </c>
+      <c r="G290" t="n">
+        <v>0.965</v>
+      </c>
+      <c r="H290" t="n">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>VOC</t>
+        </is>
+      </c>
+      <c r="B291" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>BICFA</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>BIC Corporation -- Dropship</t>
+        </is>
+      </c>
+      <c r="E291" t="n">
+        <v>202630</v>
+      </c>
+      <c r="F291" t="n">
+        <v>0.9872</v>
+      </c>
+      <c r="G291" t="n">
+        <v>0.9872</v>
+      </c>
+      <c r="H291" t="n">
+        <v>20292</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>VOC</t>
+        </is>
+      </c>
+      <c r="B292" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>CER43</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Central National-Gottesman Inc. - CNG (Private Brands) -- Dropship</t>
+        </is>
+      </c>
+      <c r="E292" t="n">
+        <v>202630</v>
+      </c>
+      <c r="F292" t="n">
+        <v>0.8632</v>
+      </c>
+      <c r="G292" t="n">
+        <v>0.8632</v>
+      </c>
+      <c r="H292" t="n">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>VOC</t>
+        </is>
+      </c>
+      <c r="B293" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>CNGNE</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>CNG NA CPB -- Dropship</t>
+        </is>
+      </c>
+      <c r="E293" t="n">
+        <v>202630</v>
+      </c>
+      <c r="F293" t="n">
+        <v>1</v>
+      </c>
+      <c r="G293" t="n">
+        <v>1</v>
+      </c>
+      <c r="H293" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>VOC</t>
+        </is>
+      </c>
+      <c r="B294" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>IMSZY</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>IMPRESO Inc(IMSZY) -- Dropship</t>
+        </is>
+      </c>
+      <c r="E294" t="n">
+        <v>202630</v>
+      </c>
+      <c r="F294" t="n">
+        <v>0.9791</v>
+      </c>
+      <c r="G294" t="n">
+        <v>0.9791</v>
+      </c>
+      <c r="H294" t="n">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>VOC</t>
+        </is>
+      </c>
+      <c r="B295" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>TIRG4</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>Tire Centers, LLC</t>
+        </is>
+      </c>
+      <c r="E295" t="n">
+        <v>202630</v>
+      </c>
+      <c r="F295" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="G295" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="H295" t="n">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>VOC</t>
+        </is>
+      </c>
+      <c r="B296" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>TV8OA</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>Tonal Systems, Inc. -- Dropship</t>
+        </is>
+      </c>
+      <c r="E296" t="n">
+        <v>202630</v>
+      </c>
+      <c r="F296" t="n">
+        <v>0</v>
+      </c>
+      <c r="G296" t="n">
+        <v>0</v>
+      </c>
+      <c r="H296" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>VOC</t>
+        </is>
+      </c>
+      <c r="B297" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>YX74K</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>Geneva Supply Inc. -- Dropship</t>
+        </is>
+      </c>
+      <c r="E297" t="n">
+        <v>202630</v>
+      </c>
+      <c r="F297" t="n">
+        <v>0.9436</v>
+      </c>
+      <c r="G297" t="n">
+        <v>0.9436</v>
+      </c>
+      <c r="H297" t="n">
+        <v>4118</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-refresh: add WK-31 VOC data
</commit_message>
<xml_diff>
--- a/VOC_data.xlsx
+++ b/VOC_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H297"/>
+  <dimension ref="A1:H305"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9942,6 +9942,262 @@
         <v>4118</v>
       </c>
     </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>VOC</t>
+        </is>
+      </c>
+      <c r="B298" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>0V6VN</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>JustFoodForDogs -- Dropship</t>
+        </is>
+      </c>
+      <c r="E298" t="n">
+        <v>202631</v>
+      </c>
+      <c r="F298" t="n">
+        <v>0.9669</v>
+      </c>
+      <c r="G298" t="n">
+        <v>0.9669</v>
+      </c>
+      <c r="H298" t="n">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>VOC</t>
+        </is>
+      </c>
+      <c r="B299" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>BICFA</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>BIC Corporation -- Dropship</t>
+        </is>
+      </c>
+      <c r="E299" t="n">
+        <v>202631</v>
+      </c>
+      <c r="F299" t="n">
+        <v>0.9885</v>
+      </c>
+      <c r="G299" t="n">
+        <v>0.9885</v>
+      </c>
+      <c r="H299" t="n">
+        <v>21314</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>VOC</t>
+        </is>
+      </c>
+      <c r="B300" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>CER43</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>Central National-Gottesman Inc. - CNG (Private Brands) -- Dropship</t>
+        </is>
+      </c>
+      <c r="E300" t="n">
+        <v>202631</v>
+      </c>
+      <c r="F300" t="n">
+        <v>0.9347</v>
+      </c>
+      <c r="G300" t="n">
+        <v>0.9347</v>
+      </c>
+      <c r="H300" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>VOC</t>
+        </is>
+      </c>
+      <c r="B301" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>CNGNE</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>CNG NA CPB -- Dropship</t>
+        </is>
+      </c>
+      <c r="E301" t="n">
+        <v>202631</v>
+      </c>
+      <c r="F301" t="n">
+        <v>0</v>
+      </c>
+      <c r="G301" t="n">
+        <v>0</v>
+      </c>
+      <c r="H301" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>VOC</t>
+        </is>
+      </c>
+      <c r="B302" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>IMSZY</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>IMPRESO Inc(IMSZY) -- Dropship</t>
+        </is>
+      </c>
+      <c r="E302" t="n">
+        <v>202631</v>
+      </c>
+      <c r="F302" t="n">
+        <v>1</v>
+      </c>
+      <c r="G302" t="n">
+        <v>1</v>
+      </c>
+      <c r="H302" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>VOC</t>
+        </is>
+      </c>
+      <c r="B303" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>TIRG4</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>Tire Centers, LLC</t>
+        </is>
+      </c>
+      <c r="E303" t="n">
+        <v>202631</v>
+      </c>
+      <c r="F303" t="n">
+        <v>0.8333</v>
+      </c>
+      <c r="G303" t="n">
+        <v>0.8333</v>
+      </c>
+      <c r="H303" t="n">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>VOC</t>
+        </is>
+      </c>
+      <c r="B304" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>TV8OA</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>Tonal Systems, Inc. -- Dropship</t>
+        </is>
+      </c>
+      <c r="E304" t="n">
+        <v>202631</v>
+      </c>
+      <c r="F304" t="n">
+        <v>1</v>
+      </c>
+      <c r="G304" t="n">
+        <v>1</v>
+      </c>
+      <c r="H304" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>VOC</t>
+        </is>
+      </c>
+      <c r="B305" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>YX74K</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>Geneva Supply Inc. -- Dropship</t>
+        </is>
+      </c>
+      <c r="E305" t="n">
+        <v>202631</v>
+      </c>
+      <c r="F305" t="n">
+        <v>0.9703000000000001</v>
+      </c>
+      <c r="G305" t="n">
+        <v>0.9703000000000001</v>
+      </c>
+      <c r="H305" t="n">
+        <v>3441</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto-refresh: add WK-32 VOC data
</commit_message>
<xml_diff>
--- a/VOC_data.xlsx
+++ b/VOC_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H305"/>
+  <dimension ref="A1:H314"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10198,6 +10198,294 @@
         <v>3441</v>
       </c>
     </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>VOC</t>
+        </is>
+      </c>
+      <c r="B306" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>0V6VN</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>JustFoodForDogs -- Dropship</t>
+        </is>
+      </c>
+      <c r="E306" t="n">
+        <v>202632</v>
+      </c>
+      <c r="F306" t="n">
+        <v>0.9315</v>
+      </c>
+      <c r="G306" t="n">
+        <v>0.9315</v>
+      </c>
+      <c r="H306" t="n">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>VOC</t>
+        </is>
+      </c>
+      <c r="B307" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>BICFA</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>BIC Corporation -- Dropship</t>
+        </is>
+      </c>
+      <c r="E307" t="n">
+        <v>202632</v>
+      </c>
+      <c r="F307" t="n">
+        <v>0.9727</v>
+      </c>
+      <c r="G307" t="n">
+        <v>0.9727</v>
+      </c>
+      <c r="H307" t="n">
+        <v>21254</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>VOC</t>
+        </is>
+      </c>
+      <c r="B308" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>CER43</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>Central National-Gottesman Inc. - CNG (Private Brands) -- Dropship</t>
+        </is>
+      </c>
+      <c r="E308" t="n">
+        <v>202632</v>
+      </c>
+      <c r="F308" t="n">
+        <v>0.7745</v>
+      </c>
+      <c r="G308" t="n">
+        <v>0.7745</v>
+      </c>
+      <c r="H308" t="n">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>VOC</t>
+        </is>
+      </c>
+      <c r="B309" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>CNGNE</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>CNG NA CPB -- Dropship</t>
+        </is>
+      </c>
+      <c r="E309" t="n">
+        <v>202632</v>
+      </c>
+      <c r="F309" t="n">
+        <v>1</v>
+      </c>
+      <c r="G309" t="n">
+        <v>1</v>
+      </c>
+      <c r="H309" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>VOC</t>
+        </is>
+      </c>
+      <c r="B310" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>IMSZY</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>IMPRESO Inc(IMSZY) -- Dropship</t>
+        </is>
+      </c>
+      <c r="E310" t="n">
+        <v>202632</v>
+      </c>
+      <c r="F310" t="n">
+        <v>0.824</v>
+      </c>
+      <c r="G310" t="n">
+        <v>0.824</v>
+      </c>
+      <c r="H310" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>VOC</t>
+        </is>
+      </c>
+      <c r="B311" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>SUW37</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>Sunrise Global Marketing - DROPSHIP</t>
+        </is>
+      </c>
+      <c r="E311" t="n">
+        <v>202632</v>
+      </c>
+      <c r="F311" t="n">
+        <v>0</v>
+      </c>
+      <c r="G311" t="n">
+        <v>0</v>
+      </c>
+      <c r="H311" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>VOC</t>
+        </is>
+      </c>
+      <c r="B312" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>TIRG4</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>Tire Centers, LLC</t>
+        </is>
+      </c>
+      <c r="E312" t="n">
+        <v>202632</v>
+      </c>
+      <c r="F312" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="G312" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="H312" t="n">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>VOC</t>
+        </is>
+      </c>
+      <c r="B313" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>TV8OA</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>Tonal Systems, Inc. -- Dropship</t>
+        </is>
+      </c>
+      <c r="E313" t="n">
+        <v>202632</v>
+      </c>
+      <c r="F313" t="n">
+        <v>0</v>
+      </c>
+      <c r="G313" t="n">
+        <v>0</v>
+      </c>
+      <c r="H313" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>VOC</t>
+        </is>
+      </c>
+      <c r="B314" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>YX74K</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>Geneva Supply Inc. -- Dropship</t>
+        </is>
+      </c>
+      <c r="E314" t="n">
+        <v>202632</v>
+      </c>
+      <c r="F314" t="n">
+        <v>0.9452</v>
+      </c>
+      <c r="G314" t="n">
+        <v>0.9452</v>
+      </c>
+      <c r="H314" t="n">
+        <v>3769</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto-refresh: add WK-35 VOC data
</commit_message>
<xml_diff>
--- a/VOC_data.xlsx
+++ b/VOC_data.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="998" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1019" uniqueCount="31">
   <si>
     <t>Wbr Carrier Group</t>
   </si>
@@ -464,7 +464,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H331"/>
+  <dimension ref="A1:H338"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -9073,6 +9073,188 @@
         <v>3800</v>
       </c>
     </row>
+    <row r="332" spans="1:8">
+      <c r="A332" t="s">
+        <v>8</v>
+      </c>
+      <c r="B332">
+        <v>2026</v>
+      </c>
+      <c r="C332" t="s">
+        <v>9</v>
+      </c>
+      <c r="D332" t="s">
+        <v>20</v>
+      </c>
+      <c r="E332">
+        <v>202635</v>
+      </c>
+      <c r="F332">
+        <v>0.9387</v>
+      </c>
+      <c r="G332">
+        <v>0.9387</v>
+      </c>
+      <c r="H332">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="333" spans="1:8">
+      <c r="A333" t="s">
+        <v>8</v>
+      </c>
+      <c r="B333">
+        <v>2026</v>
+      </c>
+      <c r="C333" t="s">
+        <v>10</v>
+      </c>
+      <c r="D333" t="s">
+        <v>21</v>
+      </c>
+      <c r="E333">
+        <v>202635</v>
+      </c>
+      <c r="F333">
+        <v>0.9679</v>
+      </c>
+      <c r="G333">
+        <v>0.9679</v>
+      </c>
+      <c r="H333">
+        <v>18205</v>
+      </c>
+    </row>
+    <row r="334" spans="1:8">
+      <c r="A334" t="s">
+        <v>8</v>
+      </c>
+      <c r="B334">
+        <v>2026</v>
+      </c>
+      <c r="C334" t="s">
+        <v>11</v>
+      </c>
+      <c r="D334" t="s">
+        <v>22</v>
+      </c>
+      <c r="E334">
+        <v>202635</v>
+      </c>
+      <c r="F334">
+        <v>0.9041</v>
+      </c>
+      <c r="G334">
+        <v>0.9041</v>
+      </c>
+      <c r="H334">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="335" spans="1:8">
+      <c r="A335" t="s">
+        <v>8</v>
+      </c>
+      <c r="B335">
+        <v>2026</v>
+      </c>
+      <c r="C335" t="s">
+        <v>12</v>
+      </c>
+      <c r="D335" t="s">
+        <v>23</v>
+      </c>
+      <c r="E335">
+        <v>202635</v>
+      </c>
+      <c r="F335">
+        <v>0</v>
+      </c>
+      <c r="G335">
+        <v>0</v>
+      </c>
+      <c r="H335">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="336" spans="1:8">
+      <c r="A336" t="s">
+        <v>8</v>
+      </c>
+      <c r="B336">
+        <v>2026</v>
+      </c>
+      <c r="C336" t="s">
+        <v>13</v>
+      </c>
+      <c r="D336" t="s">
+        <v>24</v>
+      </c>
+      <c r="E336">
+        <v>202635</v>
+      </c>
+      <c r="F336">
+        <v>0.98</v>
+      </c>
+      <c r="G336">
+        <v>0.98</v>
+      </c>
+      <c r="H336">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="337" spans="1:8">
+      <c r="A337" t="s">
+        <v>8</v>
+      </c>
+      <c r="B337">
+        <v>2026</v>
+      </c>
+      <c r="C337" t="s">
+        <v>15</v>
+      </c>
+      <c r="D337" t="s">
+        <v>26</v>
+      </c>
+      <c r="E337">
+        <v>202635</v>
+      </c>
+      <c r="F337">
+        <v>0.9607</v>
+      </c>
+      <c r="G337">
+        <v>0.9607</v>
+      </c>
+      <c r="H337">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="338" spans="1:8">
+      <c r="A338" t="s">
+        <v>8</v>
+      </c>
+      <c r="B338">
+        <v>2026</v>
+      </c>
+      <c r="C338" t="s">
+        <v>17</v>
+      </c>
+      <c r="D338" t="s">
+        <v>28</v>
+      </c>
+      <c r="E338">
+        <v>202635</v>
+      </c>
+      <c r="F338">
+        <v>0.958</v>
+      </c>
+      <c r="G338">
+        <v>0.958</v>
+      </c>
+      <c r="H338">
+        <v>3285</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add WK-36 and WK-37 VOC data
</commit_message>
<xml_diff>
--- a/VOC_data.xlsx
+++ b/VOC_data.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1019" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1067" uniqueCount="31">
   <si>
     <t>Wbr Carrier Group</t>
   </si>
@@ -464,7 +464,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H338"/>
+  <dimension ref="A1:H354"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -9255,6 +9255,422 @@
         <v>3285</v>
       </c>
     </row>
+    <row r="339" spans="1:8">
+      <c r="A339" t="s">
+        <v>8</v>
+      </c>
+      <c r="B339">
+        <v>2026</v>
+      </c>
+      <c r="C339" t="s">
+        <v>9</v>
+      </c>
+      <c r="D339" t="s">
+        <v>20</v>
+      </c>
+      <c r="E339">
+        <v>202636</v>
+      </c>
+      <c r="F339">
+        <v>0.9265</v>
+      </c>
+      <c r="G339">
+        <v>0.9265</v>
+      </c>
+      <c r="H339">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="340" spans="1:8">
+      <c r="A340" t="s">
+        <v>8</v>
+      </c>
+      <c r="B340">
+        <v>2026</v>
+      </c>
+      <c r="C340" t="s">
+        <v>10</v>
+      </c>
+      <c r="D340" t="s">
+        <v>21</v>
+      </c>
+      <c r="E340">
+        <v>202636</v>
+      </c>
+      <c r="F340">
+        <v>0.9631</v>
+      </c>
+      <c r="G340">
+        <v>0.9631</v>
+      </c>
+      <c r="H340">
+        <v>16784</v>
+      </c>
+    </row>
+    <row r="341" spans="1:8">
+      <c r="A341" t="s">
+        <v>8</v>
+      </c>
+      <c r="B341">
+        <v>2026</v>
+      </c>
+      <c r="C341" t="s">
+        <v>11</v>
+      </c>
+      <c r="D341" t="s">
+        <v>22</v>
+      </c>
+      <c r="E341">
+        <v>202636</v>
+      </c>
+      <c r="F341">
+        <v>0.8434295081967214</v>
+      </c>
+      <c r="G341">
+        <v>0.8434295081967214</v>
+      </c>
+      <c r="H341">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="342" spans="1:8">
+      <c r="A342" t="s">
+        <v>8</v>
+      </c>
+      <c r="B342">
+        <v>2026</v>
+      </c>
+      <c r="C342" t="s">
+        <v>12</v>
+      </c>
+      <c r="D342" t="s">
+        <v>23</v>
+      </c>
+      <c r="E342">
+        <v>202636</v>
+      </c>
+      <c r="F342">
+        <v>0</v>
+      </c>
+      <c r="G342">
+        <v>0</v>
+      </c>
+      <c r="H342">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="343" spans="1:8">
+      <c r="A343" t="s">
+        <v>8</v>
+      </c>
+      <c r="B343">
+        <v>2026</v>
+      </c>
+      <c r="C343" t="s">
+        <v>13</v>
+      </c>
+      <c r="D343" t="s">
+        <v>24</v>
+      </c>
+      <c r="E343">
+        <v>202636</v>
+      </c>
+      <c r="F343">
+        <v>0.9258999999999999</v>
+      </c>
+      <c r="G343">
+        <v>0.9258999999999999</v>
+      </c>
+      <c r="H343">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="344" spans="1:8">
+      <c r="A344" t="s">
+        <v>8</v>
+      </c>
+      <c r="B344">
+        <v>2026</v>
+      </c>
+      <c r="C344" t="s">
+        <v>15</v>
+      </c>
+      <c r="D344" t="s">
+        <v>26</v>
+      </c>
+      <c r="E344">
+        <v>202636</v>
+      </c>
+      <c r="F344">
+        <v>0.6587393700787402</v>
+      </c>
+      <c r="G344">
+        <v>0.6587393700787402</v>
+      </c>
+      <c r="H344">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="345" spans="1:8">
+      <c r="A345" t="s">
+        <v>8</v>
+      </c>
+      <c r="B345">
+        <v>2026</v>
+      </c>
+      <c r="C345" t="s">
+        <v>16</v>
+      </c>
+      <c r="D345" t="s">
+        <v>27</v>
+      </c>
+      <c r="E345">
+        <v>202636</v>
+      </c>
+      <c r="F345">
+        <v>0</v>
+      </c>
+      <c r="G345">
+        <v>0</v>
+      </c>
+      <c r="H345">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="346" spans="1:8">
+      <c r="A346" t="s">
+        <v>8</v>
+      </c>
+      <c r="B346">
+        <v>2026</v>
+      </c>
+      <c r="C346" t="s">
+        <v>17</v>
+      </c>
+      <c r="D346" t="s">
+        <v>28</v>
+      </c>
+      <c r="E346">
+        <v>202636</v>
+      </c>
+      <c r="F346">
+        <v>0.9324157395201688</v>
+      </c>
+      <c r="G346">
+        <v>0.9324157395201688</v>
+      </c>
+      <c r="H346">
+        <v>3793</v>
+      </c>
+    </row>
+    <row r="347" spans="1:8">
+      <c r="A347" t="s">
+        <v>8</v>
+      </c>
+      <c r="B347">
+        <v>2026</v>
+      </c>
+      <c r="C347" t="s">
+        <v>9</v>
+      </c>
+      <c r="D347" t="s">
+        <v>20</v>
+      </c>
+      <c r="E347">
+        <v>202637</v>
+      </c>
+      <c r="F347">
+        <v>0.9102</v>
+      </c>
+      <c r="G347">
+        <v>0.9102</v>
+      </c>
+      <c r="H347">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="348" spans="1:8">
+      <c r="A348" t="s">
+        <v>8</v>
+      </c>
+      <c r="B348">
+        <v>2026</v>
+      </c>
+      <c r="C348" t="s">
+        <v>10</v>
+      </c>
+      <c r="D348" t="s">
+        <v>21</v>
+      </c>
+      <c r="E348">
+        <v>202637</v>
+      </c>
+      <c r="F348">
+        <v>0.9967</v>
+      </c>
+      <c r="G348">
+        <v>0.9967</v>
+      </c>
+      <c r="H348">
+        <v>21490</v>
+      </c>
+    </row>
+    <row r="349" spans="1:8">
+      <c r="A349" t="s">
+        <v>8</v>
+      </c>
+      <c r="B349">
+        <v>2026</v>
+      </c>
+      <c r="C349" t="s">
+        <v>11</v>
+      </c>
+      <c r="D349" t="s">
+        <v>22</v>
+      </c>
+      <c r="E349">
+        <v>202637</v>
+      </c>
+      <c r="F349">
+        <v>1</v>
+      </c>
+      <c r="G349">
+        <v>1</v>
+      </c>
+      <c r="H349">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="350" spans="1:8">
+      <c r="A350" t="s">
+        <v>8</v>
+      </c>
+      <c r="B350">
+        <v>2026</v>
+      </c>
+      <c r="C350" t="s">
+        <v>12</v>
+      </c>
+      <c r="D350" t="s">
+        <v>23</v>
+      </c>
+      <c r="E350">
+        <v>202637</v>
+      </c>
+      <c r="F350">
+        <v>0</v>
+      </c>
+      <c r="G350">
+        <v>0</v>
+      </c>
+      <c r="H350">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="351" spans="1:8">
+      <c r="A351" t="s">
+        <v>8</v>
+      </c>
+      <c r="B351">
+        <v>2026</v>
+      </c>
+      <c r="C351" t="s">
+        <v>13</v>
+      </c>
+      <c r="D351" t="s">
+        <v>24</v>
+      </c>
+      <c r="E351">
+        <v>202637</v>
+      </c>
+      <c r="F351">
+        <v>1</v>
+      </c>
+      <c r="G351">
+        <v>1</v>
+      </c>
+      <c r="H351">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="352" spans="1:8">
+      <c r="A352" t="s">
+        <v>8</v>
+      </c>
+      <c r="B352">
+        <v>2026</v>
+      </c>
+      <c r="C352" t="s">
+        <v>15</v>
+      </c>
+      <c r="D352" t="s">
+        <v>26</v>
+      </c>
+      <c r="E352">
+        <v>202637</v>
+      </c>
+      <c r="F352">
+        <v>0.0579272727272727</v>
+      </c>
+      <c r="G352">
+        <v>0.0579272727272727</v>
+      </c>
+      <c r="H352">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="353" spans="1:8">
+      <c r="A353" t="s">
+        <v>8</v>
+      </c>
+      <c r="B353">
+        <v>2026</v>
+      </c>
+      <c r="C353" t="s">
+        <v>16</v>
+      </c>
+      <c r="D353" t="s">
+        <v>27</v>
+      </c>
+      <c r="E353">
+        <v>202637</v>
+      </c>
+      <c r="F353">
+        <v>0</v>
+      </c>
+      <c r="G353">
+        <v>0</v>
+      </c>
+      <c r="H353">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="354" spans="1:8">
+      <c r="A354" t="s">
+        <v>8</v>
+      </c>
+      <c r="B354">
+        <v>2026</v>
+      </c>
+      <c r="C354" t="s">
+        <v>17</v>
+      </c>
+      <c r="D354" t="s">
+        <v>28</v>
+      </c>
+      <c r="E354">
+        <v>202637</v>
+      </c>
+      <c r="F354">
+        <v>0.9837721461187215</v>
+      </c>
+      <c r="G354">
+        <v>0.9837721461187215</v>
+      </c>
+      <c r="H354">
+        <v>3723</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto-refresh: add WK-38 VOC data
</commit_message>
<xml_diff>
--- a/VOC_data.xlsx
+++ b/VOC_data.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1067" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1091" uniqueCount="31">
   <si>
     <t>Wbr Carrier Group</t>
   </si>
@@ -464,7 +464,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H354"/>
+  <dimension ref="A1:H362"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -9671,6 +9671,214 @@
         <v>3723</v>
       </c>
     </row>
+    <row r="355" spans="1:8">
+      <c r="A355" t="s">
+        <v>8</v>
+      </c>
+      <c r="B355">
+        <v>2026</v>
+      </c>
+      <c r="C355" t="s">
+        <v>9</v>
+      </c>
+      <c r="D355" t="s">
+        <v>20</v>
+      </c>
+      <c r="E355">
+        <v>202638</v>
+      </c>
+      <c r="F355">
+        <v>0.9539</v>
+      </c>
+      <c r="G355">
+        <v>0.9539</v>
+      </c>
+      <c r="H355">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="356" spans="1:8">
+      <c r="A356" t="s">
+        <v>8</v>
+      </c>
+      <c r="B356">
+        <v>2026</v>
+      </c>
+      <c r="C356" t="s">
+        <v>10</v>
+      </c>
+      <c r="D356" t="s">
+        <v>21</v>
+      </c>
+      <c r="E356">
+        <v>202638</v>
+      </c>
+      <c r="F356">
+        <v>0.9745</v>
+      </c>
+      <c r="G356">
+        <v>0.9745</v>
+      </c>
+      <c r="H356">
+        <v>24321</v>
+      </c>
+    </row>
+    <row r="357" spans="1:8">
+      <c r="A357" t="s">
+        <v>8</v>
+      </c>
+      <c r="B357">
+        <v>2026</v>
+      </c>
+      <c r="C357" t="s">
+        <v>11</v>
+      </c>
+      <c r="D357" t="s">
+        <v>22</v>
+      </c>
+      <c r="E357">
+        <v>202638</v>
+      </c>
+      <c r="F357">
+        <v>0.8643999999999999</v>
+      </c>
+      <c r="G357">
+        <v>0.8643999999999999</v>
+      </c>
+      <c r="H357">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="358" spans="1:8">
+      <c r="A358" t="s">
+        <v>8</v>
+      </c>
+      <c r="B358">
+        <v>2026</v>
+      </c>
+      <c r="C358" t="s">
+        <v>12</v>
+      </c>
+      <c r="D358" t="s">
+        <v>23</v>
+      </c>
+      <c r="E358">
+        <v>202638</v>
+      </c>
+      <c r="F358">
+        <v>0</v>
+      </c>
+      <c r="G358">
+        <v>0</v>
+      </c>
+      <c r="H358">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="359" spans="1:8">
+      <c r="A359" t="s">
+        <v>8</v>
+      </c>
+      <c r="B359">
+        <v>2026</v>
+      </c>
+      <c r="C359" t="s">
+        <v>13</v>
+      </c>
+      <c r="D359" t="s">
+        <v>24</v>
+      </c>
+      <c r="E359">
+        <v>202638</v>
+      </c>
+      <c r="F359">
+        <v>0.9912</v>
+      </c>
+      <c r="G359">
+        <v>0.9912</v>
+      </c>
+      <c r="H359">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="360" spans="1:8">
+      <c r="A360" t="s">
+        <v>8</v>
+      </c>
+      <c r="B360">
+        <v>2026</v>
+      </c>
+      <c r="C360" t="s">
+        <v>15</v>
+      </c>
+      <c r="D360" t="s">
+        <v>26</v>
+      </c>
+      <c r="E360">
+        <v>202638</v>
+      </c>
+      <c r="F360">
+        <v>0.5294</v>
+      </c>
+      <c r="G360">
+        <v>0.5294</v>
+      </c>
+      <c r="H360">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="361" spans="1:8">
+      <c r="A361" t="s">
+        <v>8</v>
+      </c>
+      <c r="B361">
+        <v>2026</v>
+      </c>
+      <c r="C361" t="s">
+        <v>16</v>
+      </c>
+      <c r="D361" t="s">
+        <v>27</v>
+      </c>
+      <c r="E361">
+        <v>202638</v>
+      </c>
+      <c r="F361">
+        <v>0</v>
+      </c>
+      <c r="G361">
+        <v>0</v>
+      </c>
+      <c r="H361">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="362" spans="1:8">
+      <c r="A362" t="s">
+        <v>8</v>
+      </c>
+      <c r="B362">
+        <v>2026</v>
+      </c>
+      <c r="C362" t="s">
+        <v>17</v>
+      </c>
+      <c r="D362" t="s">
+        <v>28</v>
+      </c>
+      <c r="E362">
+        <v>202638</v>
+      </c>
+      <c r="F362">
+        <v>0.9560999999999999</v>
+      </c>
+      <c r="G362">
+        <v>0.9560999999999999</v>
+      </c>
+      <c r="H362">
+        <v>3950</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto-refresh: add WK-42 VOC data
</commit_message>
<xml_diff>
--- a/VOC_data.xlsx
+++ b/VOC_data.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1091" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1112" uniqueCount="31">
   <si>
     <t>Wbr Carrier Group</t>
   </si>
@@ -464,7 +464,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H362"/>
+  <dimension ref="A1:H369"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -9879,6 +9879,188 @@
         <v>3950</v>
       </c>
     </row>
+    <row r="363" spans="1:8">
+      <c r="A363" t="s">
+        <v>8</v>
+      </c>
+      <c r="B363">
+        <v>2026</v>
+      </c>
+      <c r="C363" t="s">
+        <v>9</v>
+      </c>
+      <c r="D363" t="s">
+        <v>20</v>
+      </c>
+      <c r="E363">
+        <v>202642</v>
+      </c>
+      <c r="F363">
+        <v>0.765</v>
+      </c>
+      <c r="G363">
+        <v>0.765</v>
+      </c>
+      <c r="H363">
+        <v>590</v>
+      </c>
+    </row>
+    <row r="364" spans="1:8">
+      <c r="A364" t="s">
+        <v>8</v>
+      </c>
+      <c r="B364">
+        <v>2026</v>
+      </c>
+      <c r="C364" t="s">
+        <v>10</v>
+      </c>
+      <c r="D364" t="s">
+        <v>21</v>
+      </c>
+      <c r="E364">
+        <v>202642</v>
+      </c>
+      <c r="F364">
+        <v>0.987</v>
+      </c>
+      <c r="G364">
+        <v>0.987</v>
+      </c>
+      <c r="H364">
+        <v>22295</v>
+      </c>
+    </row>
+    <row r="365" spans="1:8">
+      <c r="A365" t="s">
+        <v>8</v>
+      </c>
+      <c r="B365">
+        <v>2026</v>
+      </c>
+      <c r="C365" t="s">
+        <v>11</v>
+      </c>
+      <c r="D365" t="s">
+        <v>22</v>
+      </c>
+      <c r="E365">
+        <v>202642</v>
+      </c>
+      <c r="F365">
+        <v>1</v>
+      </c>
+      <c r="G365">
+        <v>1</v>
+      </c>
+      <c r="H365">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="366" spans="1:8">
+      <c r="A366" t="s">
+        <v>8</v>
+      </c>
+      <c r="B366">
+        <v>2026</v>
+      </c>
+      <c r="C366" t="s">
+        <v>12</v>
+      </c>
+      <c r="D366" t="s">
+        <v>23</v>
+      </c>
+      <c r="E366">
+        <v>202642</v>
+      </c>
+      <c r="F366">
+        <v>0</v>
+      </c>
+      <c r="G366">
+        <v>0</v>
+      </c>
+      <c r="H366">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="367" spans="1:8">
+      <c r="A367" t="s">
+        <v>8</v>
+      </c>
+      <c r="B367">
+        <v>2026</v>
+      </c>
+      <c r="C367" t="s">
+        <v>13</v>
+      </c>
+      <c r="D367" t="s">
+        <v>24</v>
+      </c>
+      <c r="E367">
+        <v>202642</v>
+      </c>
+      <c r="F367">
+        <v>1</v>
+      </c>
+      <c r="G367">
+        <v>1</v>
+      </c>
+      <c r="H367">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="368" spans="1:8">
+      <c r="A368" t="s">
+        <v>8</v>
+      </c>
+      <c r="B368">
+        <v>2026</v>
+      </c>
+      <c r="C368" t="s">
+        <v>15</v>
+      </c>
+      <c r="D368" t="s">
+        <v>26</v>
+      </c>
+      <c r="E368">
+        <v>202642</v>
+      </c>
+      <c r="F368">
+        <v>0.9213</v>
+      </c>
+      <c r="G368">
+        <v>0.9213</v>
+      </c>
+      <c r="H368">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="369" spans="1:8">
+      <c r="A369" t="s">
+        <v>8</v>
+      </c>
+      <c r="B369">
+        <v>2026</v>
+      </c>
+      <c r="C369" t="s">
+        <v>17</v>
+      </c>
+      <c r="D369" t="s">
+        <v>28</v>
+      </c>
+      <c r="E369">
+        <v>202642</v>
+      </c>
+      <c r="F369">
+        <v>0.9811</v>
+      </c>
+      <c r="G369">
+        <v>0.9811</v>
+      </c>
+      <c r="H369">
+        <v>2604</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto-refresh: add WK-43 VOC data
</commit_message>
<xml_diff>
--- a/VOC_data.xlsx
+++ b/VOC_data.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1112" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1130" uniqueCount="31">
   <si>
     <t>Wbr Carrier Group</t>
   </si>
@@ -464,7 +464,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H369"/>
+  <dimension ref="A1:H375"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -10061,6 +10061,162 @@
         <v>2604</v>
       </c>
     </row>
+    <row r="370" spans="1:8">
+      <c r="A370" t="s">
+        <v>8</v>
+      </c>
+      <c r="B370">
+        <v>2026</v>
+      </c>
+      <c r="C370" t="s">
+        <v>9</v>
+      </c>
+      <c r="D370" t="s">
+        <v>20</v>
+      </c>
+      <c r="E370">
+        <v>202643</v>
+      </c>
+      <c r="F370">
+        <v>0.95</v>
+      </c>
+      <c r="G370">
+        <v>0.95</v>
+      </c>
+      <c r="H370">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="371" spans="1:8">
+      <c r="A371" t="s">
+        <v>8</v>
+      </c>
+      <c r="B371">
+        <v>2026</v>
+      </c>
+      <c r="C371" t="s">
+        <v>10</v>
+      </c>
+      <c r="D371" t="s">
+        <v>21</v>
+      </c>
+      <c r="E371">
+        <v>202643</v>
+      </c>
+      <c r="F371">
+        <v>0.9832</v>
+      </c>
+      <c r="G371">
+        <v>0.9832</v>
+      </c>
+      <c r="H371">
+        <v>19823</v>
+      </c>
+    </row>
+    <row r="372" spans="1:8">
+      <c r="A372" t="s">
+        <v>8</v>
+      </c>
+      <c r="B372">
+        <v>2026</v>
+      </c>
+      <c r="C372" t="s">
+        <v>11</v>
+      </c>
+      <c r="D372" t="s">
+        <v>22</v>
+      </c>
+      <c r="E372">
+        <v>202643</v>
+      </c>
+      <c r="F372">
+        <v>0.9764</v>
+      </c>
+      <c r="G372">
+        <v>0.9764</v>
+      </c>
+      <c r="H372">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="373" spans="1:8">
+      <c r="A373" t="s">
+        <v>8</v>
+      </c>
+      <c r="B373">
+        <v>2026</v>
+      </c>
+      <c r="C373" t="s">
+        <v>13</v>
+      </c>
+      <c r="D373" t="s">
+        <v>24</v>
+      </c>
+      <c r="E373">
+        <v>202643</v>
+      </c>
+      <c r="F373">
+        <v>1</v>
+      </c>
+      <c r="G373">
+        <v>1</v>
+      </c>
+      <c r="H373">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="374" spans="1:8">
+      <c r="A374" t="s">
+        <v>8</v>
+      </c>
+      <c r="B374">
+        <v>2026</v>
+      </c>
+      <c r="C374" t="s">
+        <v>15</v>
+      </c>
+      <c r="D374" t="s">
+        <v>26</v>
+      </c>
+      <c r="E374">
+        <v>202643</v>
+      </c>
+      <c r="F374">
+        <v>0.9114</v>
+      </c>
+      <c r="G374">
+        <v>0.9114</v>
+      </c>
+      <c r="H374">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="375" spans="1:8">
+      <c r="A375" t="s">
+        <v>8</v>
+      </c>
+      <c r="B375">
+        <v>2026</v>
+      </c>
+      <c r="C375" t="s">
+        <v>17</v>
+      </c>
+      <c r="D375" t="s">
+        <v>28</v>
+      </c>
+      <c r="E375">
+        <v>202643</v>
+      </c>
+      <c r="F375">
+        <v>0.9917</v>
+      </c>
+      <c r="G375">
+        <v>0.9917</v>
+      </c>
+      <c r="H375">
+        <v>3157</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>